<commit_message>
Rename com.flowpay to com.payflow, show rollback stages in payment history, add combined Docker image
</commit_message>
<xml_diff>
--- a/04_Client_Feedback_Decision_Log.xlsx
+++ b/04_Client_Feedback_Decision_Log.xlsx
@@ -1,19 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Client Feedback Log" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Decision Log" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="Client Feedback Log" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="Decision Log" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
-  <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Client Feedback Log'!$A$1:$F$4</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Decision Log'!$A$1:$F$4</definedName>
-  </definedNames>
+  <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
 </file>
@@ -44,7 +41,6 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="001F4E78"/>
-        <bgColor rgb="001F4E78"/>
       </patternFill>
     </fill>
   </fills>
@@ -57,10 +53,18 @@
       <diagonal/>
     </border>
     <border>
-      <left style="thin"/>
-      <right style="thin"/>
-      <top style="thin"/>
-      <bottom style="thin"/>
+      <left style="thin">
+        <color rgb="00B7B7B7"/>
+      </left>
+      <right style="thin">
+        <color rgb="00B7B7B7"/>
+      </right>
+      <top style="thin">
+        <color rgb="00B7B7B7"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="00B7B7B7"/>
+      </bottom>
     </border>
   </borders>
   <cellStyleXfs count="1">
@@ -69,7 +73,7 @@
   <cellXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center"/>
+      <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
@@ -439,15 +443,16 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F4"/>
+  <dimension ref="A1:G11"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="10" customWidth="1" min="1" max="1"/>
-    <col width="13" customWidth="1" min="2" max="2"/>
-    <col width="50" customWidth="1" min="3" max="3"/>
-    <col width="10" customWidth="1" min="4" max="4"/>
-    <col width="13" customWidth="1" min="5" max="5"/>
-    <col width="48" customWidth="1" min="6" max="6"/>
+    <col width="12" customWidth="1" min="1" max="1"/>
+    <col width="14" customWidth="1" min="2" max="2"/>
+    <col width="26" customWidth="1" min="3" max="3"/>
+    <col width="60" customWidth="1" min="4" max="4"/>
+    <col width="11" customWidth="1" min="5" max="5"/>
+    <col width="14" customWidth="1" min="6" max="6"/>
+    <col width="55" customWidth="1" min="7" max="7"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -463,22 +468,27 @@
       </c>
       <c r="C1" s="1" t="inlineStr">
         <is>
+          <t>Related Epic</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
           <t>Feedback</t>
         </is>
       </c>
-      <c r="D1" s="1" t="inlineStr">
+      <c r="E1" s="1" t="inlineStr">
         <is>
           <t>Priority</t>
         </is>
       </c>
-      <c r="E1" s="1" t="inlineStr">
+      <c r="F1" s="1" t="inlineStr">
         <is>
           <t>Assigned To</t>
         </is>
       </c>
-      <c r="F1" s="1" t="inlineStr">
-        <is>
-          <t>Status</t>
+      <c r="G1" s="1" t="inlineStr">
+        <is>
+          <t>Status / Outcome</t>
         </is>
       </c>
     </row>
@@ -490,27 +500,32 @@
       </c>
       <c r="B2" s="2" t="inlineStr">
         <is>
-          <t>01-Aug-2026</t>
+          <t>29-Jul-2026</t>
         </is>
       </c>
       <c r="C2" s="2" t="inlineStr">
         <is>
-          <t>Ensure security user login utilizes strong hashing before DB insertion.</t>
+          <t>Authentication &amp; Security</t>
         </is>
       </c>
       <c r="D2" s="2" t="inlineStr">
         <is>
+          <t>Ensure user login uses strong password hashing and stateless auth so the API scales without server-side sessions.</t>
+        </is>
+      </c>
+      <c r="E2" s="2" t="inlineStr">
+        <is>
           <t>High</t>
         </is>
       </c>
-      <c r="E2" s="2" t="inlineStr">
-        <is>
-          <t>Anusree</t>
-        </is>
-      </c>
       <c r="F2" s="2" t="inlineStr">
         <is>
-          <t>Implemented in Sprint 2</t>
+          <t>Dhruv</t>
+        </is>
+      </c>
+      <c r="G2" s="2" t="inlineStr">
+        <is>
+          <t>Implemented - JWT auth + BCrypt hashing (JwtAuthFilter, SecurityConfig)</t>
         </is>
       </c>
     </row>
@@ -527,59 +542,327 @@
       </c>
       <c r="C3" s="2" t="inlineStr">
         <is>
+          <t>Payment Processing</t>
+        </is>
+      </c>
+      <c r="D3" s="2" t="inlineStr">
+        <is>
           <t>Need support for multiple payment methods, not just bank transfer.</t>
         </is>
       </c>
-      <c r="D3" s="2" t="inlineStr">
+      <c r="E3" s="2" t="inlineStr">
         <is>
           <t>Medium</t>
         </is>
       </c>
-      <c r="E3" s="2" t="inlineStr">
+      <c r="F3" s="2" t="inlineStr">
         <is>
           <t>Dhruv</t>
         </is>
       </c>
-      <c r="F3" s="2" t="inlineStr">
-        <is>
-          <t>Added PaymentMethod enum to model</t>
+      <c r="G3" s="2" t="inlineStr">
+        <is>
+          <t>Implemented - PaymentMethod enum added to Payment model</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="2" t="inlineStr">
         <is>
+          <t>Sprint 2</t>
+        </is>
+      </c>
+      <c r="B4" s="2" t="inlineStr">
+        <is>
+          <t>02-Aug-2026</t>
+        </is>
+      </c>
+      <c r="C4" s="2" t="inlineStr">
+        <is>
+          <t>Payment Processing</t>
+        </is>
+      </c>
+      <c r="D4" s="2" t="inlineStr">
+        <is>
+          <t>Sensitive account details must be protected at rest, not just in transit.</t>
+        </is>
+      </c>
+      <c r="E4" s="2" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="F4" s="2" t="inlineStr">
+        <is>
+          <t>Anusree</t>
+        </is>
+      </c>
+      <c r="G4" s="2" t="inlineStr">
+        <is>
+          <t>Implemented - encryption added for account details in payment service</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="2" t="inlineStr">
+        <is>
+          <t>Sprint 3</t>
+        </is>
+      </c>
+      <c r="B5" s="2" t="inlineStr">
+        <is>
+          <t>03-Aug-2026</t>
+        </is>
+      </c>
+      <c r="C5" s="2" t="inlineStr">
+        <is>
+          <t>DevOps &amp; Infrastructure</t>
+        </is>
+      </c>
+      <c r="D5" s="2" t="inlineStr">
+        <is>
+          <t>Application should be easy to run consistently across environments for demos and grading.</t>
+        </is>
+      </c>
+      <c r="E5" s="2" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="F5" s="2" t="inlineStr">
+        <is>
+          <t>Dhruv</t>
+        </is>
+      </c>
+      <c r="G5" s="2" t="inlineStr">
+        <is>
+          <t>Implemented - Dockerfile (backend/frontend) + docker-compose.yml</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="2" t="inlineStr">
+        <is>
+          <t>Sprint 3</t>
+        </is>
+      </c>
+      <c r="B6" s="2" t="inlineStr">
+        <is>
+          <t>03-Aug-2026</t>
+        </is>
+      </c>
+      <c r="C6" s="2" t="inlineStr">
+        <is>
+          <t>Testing &amp; Quality Assurance</t>
+        </is>
+      </c>
+      <c r="D6" s="2" t="inlineStr">
+        <is>
+          <t>Core auth and payment logic needs automated test coverage before further features are layered on top.</t>
+        </is>
+      </c>
+      <c r="E6" s="2" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="F6" s="2" t="inlineStr">
+        <is>
+          <t>Anusree</t>
+        </is>
+      </c>
+      <c r="G6" s="2" t="inlineStr">
+        <is>
+          <t>Implemented - unit tests for auth and payment service</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="2" t="inlineStr">
+        <is>
           <t>Sprint 4</t>
         </is>
       </c>
-      <c r="B4" s="2" t="inlineStr">
+      <c r="B7" s="2" t="inlineStr">
         <is>
           <t>04-Aug-2026</t>
         </is>
       </c>
-      <c r="C4" s="2" t="inlineStr">
-        <is>
-          <t>Payment history must explicitly show failed transactions and handle rollback cleanly.</t>
-        </is>
-      </c>
-      <c r="D4" s="2" t="inlineStr">
+      <c r="C7" s="2" t="inlineStr">
+        <is>
+          <t>Payment Processing</t>
+        </is>
+      </c>
+      <c r="D7" s="2" t="inlineStr">
+        <is>
+          <t>Payment history must explicitly show failed transactions and handle rollback cleanly, with the money visibly returned.</t>
+        </is>
+      </c>
+      <c r="E7" s="2" t="inlineStr">
         <is>
           <t>Critical</t>
         </is>
       </c>
-      <c r="E4" s="2" t="inlineStr">
+      <c r="F7" s="2" t="inlineStr">
+        <is>
+          <t>Dhruv</t>
+        </is>
+      </c>
+      <c r="G7" s="2" t="inlineStr">
+        <is>
+          <t>Implemented - deterministic failure simulation + automatic refund/rollback + audit history logging</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="2" t="inlineStr">
+        <is>
+          <t>Sprint 4</t>
+        </is>
+      </c>
+      <c r="B8" s="2" t="inlineStr">
+        <is>
+          <t>04-Aug-2026</t>
+        </is>
+      </c>
+      <c r="C8" s="2" t="inlineStr">
+        <is>
+          <t>Payment Processing</t>
+        </is>
+      </c>
+      <c r="D8" s="2" t="inlineStr">
+        <is>
+          <t>Users should be able to search/filter their payment history by status, amount, and date.</t>
+        </is>
+      </c>
+      <c r="E8" s="2" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="F8" s="2" t="inlineStr">
+        <is>
+          <t>Dhruv</t>
+        </is>
+      </c>
+      <c r="G8" s="2" t="inlineStr">
+        <is>
+          <t>Implemented - GET /api/payments/search endpoint with status/amount/date filters</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="2" t="inlineStr">
+        <is>
+          <t>Sprint 4</t>
+        </is>
+      </c>
+      <c r="B9" s="2" t="inlineStr">
+        <is>
+          <t>04-Aug-2026</t>
+        </is>
+      </c>
+      <c r="C9" s="2" t="inlineStr">
+        <is>
+          <t>Security &amp; Authentication</t>
+        </is>
+      </c>
+      <c r="D9" s="2" t="inlineStr">
+        <is>
+          <t>Users should be able to change their own password without contacting support.</t>
+        </is>
+      </c>
+      <c r="E9" s="2" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="F9" s="2" t="inlineStr">
         <is>
           <t>Anusree</t>
         </is>
       </c>
-      <c r="F4" s="2" t="inlineStr">
-        <is>
-          <t>Implemented via PaymentHistory and TriggerType</t>
+      <c r="G9" s="2" t="inlineStr">
+        <is>
+          <t>Implemented - isolated password-change feature (reverted once, re-added cleanly) via AccountController/PasswordService</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="2" t="inlineStr">
+        <is>
+          <t>Sprint 5</t>
+        </is>
+      </c>
+      <c r="B10" s="2" t="inlineStr">
+        <is>
+          <t>05-Aug-2026</t>
+        </is>
+      </c>
+      <c r="C10" s="2" t="inlineStr">
+        <is>
+          <t>DevOps &amp; Quality</t>
+        </is>
+      </c>
+      <c r="D10" s="2" t="inlineStr">
+        <is>
+          <t>Project needs clear agile documentation (vision, epics, sprint allocation) for client/stakeholder visibility.</t>
+        </is>
+      </c>
+      <c r="E10" s="2" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="F10" s="2" t="inlineStr">
+        <is>
+          <t>Dhruv</t>
+        </is>
+      </c>
+      <c r="G10" s="2" t="inlineStr">
+        <is>
+          <t>Implemented - agile sprint documentation and architectural specs added</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="2" t="inlineStr">
+        <is>
+          <t>Sprint 5</t>
+        </is>
+      </c>
+      <c r="B11" s="2" t="inlineStr">
+        <is>
+          <t>05-Aug-2026</t>
+        </is>
+      </c>
+      <c r="C11" s="2" t="inlineStr">
+        <is>
+          <t>User Experience &amp; Frontend</t>
+        </is>
+      </c>
+      <c r="D11" s="2" t="inlineStr">
+        <is>
+          <t>Payment list page should expose the new amount/date range filters directly in the UI, not just via API.</t>
+        </is>
+      </c>
+      <c r="E11" s="2" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="F11" s="2" t="inlineStr">
+        <is>
+          <t>Chaitanya</t>
+        </is>
+      </c>
+      <c r="G11" s="2" t="inlineStr">
+        <is>
+          <t>Implemented - amount and date range filters added to Payment List page</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:F4"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -590,15 +873,16 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F4"/>
+  <dimension ref="A1:G9"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="8" customWidth="1" min="1" max="1"/>
-    <col width="13" customWidth="1" min="2" max="2"/>
-    <col width="36" customWidth="1" min="3" max="3"/>
-    <col width="50" customWidth="1" min="4" max="4"/>
+    <col width="9" customWidth="1" min="1" max="1"/>
+    <col width="11" customWidth="1" min="2" max="2"/>
+    <col width="14" customWidth="1" min="3" max="3"/>
+    <col width="46" customWidth="1" min="4" max="4"/>
     <col width="46" customWidth="1" min="5" max="5"/>
-    <col width="9" customWidth="1" min="6" max="6"/>
+    <col width="50" customWidth="1" min="6" max="6"/>
+    <col width="11" customWidth="1" min="7" max="7"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -609,25 +893,30 @@
       </c>
       <c r="B1" s="1" t="inlineStr">
         <is>
+          <t>Sprint</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
           <t>Date</t>
         </is>
       </c>
-      <c r="C1" s="1" t="inlineStr">
+      <c r="D1" s="1" t="inlineStr">
         <is>
           <t>Decision</t>
         </is>
       </c>
-      <c r="D1" s="1" t="inlineStr">
+      <c r="E1" s="1" t="inlineStr">
         <is>
           <t>Reason</t>
         </is>
       </c>
-      <c r="E1" s="1" t="inlineStr">
+      <c r="F1" s="1" t="inlineStr">
         <is>
           <t>Impact</t>
         </is>
       </c>
-      <c r="F1" s="1" t="inlineStr">
+      <c r="G1" s="1" t="inlineStr">
         <is>
           <t>Owner</t>
         </is>
@@ -641,25 +930,30 @@
       </c>
       <c r="B2" s="2" t="inlineStr">
         <is>
+          <t>Sprint 1</t>
+        </is>
+      </c>
+      <c r="C2" s="2" t="inlineStr">
+        <is>
           <t>29-Jul-2026</t>
         </is>
       </c>
-      <c r="C2" s="2" t="inlineStr">
+      <c r="D2" s="2" t="inlineStr">
         <is>
           <t>Use Spring Boot and React/Vite</t>
         </is>
       </c>
-      <c r="D2" s="2" t="inlineStr">
+      <c r="E2" s="2" t="inlineStr">
         <is>
           <t>Aligns with team expertise and project requirements</t>
         </is>
       </c>
-      <c r="E2" s="2" t="inlineStr">
-        <is>
-          <t>Determines complete tech stack</t>
-        </is>
-      </c>
       <c r="F2" s="2" t="inlineStr">
+        <is>
+          <t>Determines the complete tech stack</t>
+        </is>
+      </c>
+      <c r="G2" s="2" t="inlineStr">
         <is>
           <t>Dhruv</t>
         </is>
@@ -673,25 +967,30 @@
       </c>
       <c r="B3" s="2" t="inlineStr">
         <is>
+          <t>Sprint 1</t>
+        </is>
+      </c>
+      <c r="C3" s="2" t="inlineStr">
+        <is>
           <t>29-Jul-2026</t>
         </is>
       </c>
-      <c r="C3" s="2" t="inlineStr">
-        <is>
-          <t>Implement JWT for stateless Auth</t>
-        </is>
-      </c>
       <c r="D3" s="2" t="inlineStr">
         <is>
-          <t>Better scaling, no session state required on API</t>
+          <t>Implement JWT for stateless auth</t>
         </is>
       </c>
       <c r="E3" s="2" t="inlineStr">
         <is>
+          <t>Better scaling; no session state required on the API</t>
+        </is>
+      </c>
+      <c r="F3" s="2" t="inlineStr">
+        <is>
           <t>Requires custom JwtAuthFilter</t>
         </is>
       </c>
-      <c r="F3" s="2" t="inlineStr">
+      <c r="G3" s="2" t="inlineStr">
         <is>
           <t>Dhruv</t>
         </is>
@@ -705,32 +1004,221 @@
       </c>
       <c r="B4" s="2" t="inlineStr">
         <is>
+          <t>Sprint 2</t>
+        </is>
+      </c>
+      <c r="C4" s="2" t="inlineStr">
+        <is>
           <t>02-Aug-2026</t>
         </is>
       </c>
-      <c r="C4" s="2" t="inlineStr">
-        <is>
-          <t>Simulate external payment gateways</t>
-        </is>
-      </c>
       <c r="D4" s="2" t="inlineStr">
         <is>
-          <t>Scope restriction; real integration not required for assessment</t>
+          <t>Simulate external payment gateways instead of real integration</t>
         </is>
       </c>
       <c r="E4" s="2" t="inlineStr">
         <is>
-          <t>Created internal state transition simulation</t>
+          <t>Scope restriction; real payment gateway integration not required for assessment</t>
         </is>
       </c>
       <c r="F4" s="2" t="inlineStr">
         <is>
+          <t>Created internal state-transition simulation in PaymentService</t>
+        </is>
+      </c>
+      <c r="G4" s="2" t="inlineStr">
+        <is>
           <t>Anusree</t>
         </is>
       </c>
     </row>
+    <row r="5">
+      <c r="A5" s="2" t="inlineStr">
+        <is>
+          <t>DEC-04</t>
+        </is>
+      </c>
+      <c r="B5" s="2" t="inlineStr">
+        <is>
+          <t>Sprint 4</t>
+        </is>
+      </c>
+      <c r="C5" s="2" t="inlineStr">
+        <is>
+          <t>04-Aug-2026</t>
+        </is>
+      </c>
+      <c r="D5" s="2" t="inlineStr">
+        <is>
+          <t>Rename project package/branding from FlowPay to PayFlow</t>
+        </is>
+      </c>
+      <c r="E5" s="2" t="inlineStr">
+        <is>
+          <t>Standardize naming across team after parallel branch work created inconsistent package names</t>
+        </is>
+      </c>
+      <c r="F5" s="2" t="inlineStr">
+        <is>
+          <t>Required merging unrelated git histories (--allow-unrelated-histories) and removing leftover com.flowpay files</t>
+        </is>
+      </c>
+      <c r="G5" s="2" t="inlineStr">
+        <is>
+          <t>Dhruv</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="2" t="inlineStr">
+        <is>
+          <t>DEC-05</t>
+        </is>
+      </c>
+      <c r="B6" s="2" t="inlineStr">
+        <is>
+          <t>Sprint 4</t>
+        </is>
+      </c>
+      <c r="C6" s="2" t="inlineStr">
+        <is>
+          <t>04-Aug-2026</t>
+        </is>
+      </c>
+      <c r="D6" s="2" t="inlineStr">
+        <is>
+          <t>Make every 3rd transaction fail deterministically (instead of random)</t>
+        </is>
+      </c>
+      <c r="E6" s="2" t="inlineStr">
+        <is>
+          <t>Random success/failure was not reliably demonstrable/testable for the client demo</t>
+        </is>
+      </c>
+      <c r="F6" s="2" t="inlineStr">
+        <is>
+          <t>Added AtomicLong transactionCounter to PaymentService for repeatable, testable failure simulation</t>
+        </is>
+      </c>
+      <c r="G6" s="2" t="inlineStr">
+        <is>
+          <t>Dhruv</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="2" t="inlineStr">
+        <is>
+          <t>DEC-06</t>
+        </is>
+      </c>
+      <c r="B7" s="2" t="inlineStr">
+        <is>
+          <t>Sprint 4</t>
+        </is>
+      </c>
+      <c r="C7" s="2" t="inlineStr">
+        <is>
+          <t>04-Aug-2026</t>
+        </is>
+      </c>
+      <c r="D7" s="2" t="inlineStr">
+        <is>
+          <t>Debit funds upfront and auto-refund on failure (rollback) instead of retry</t>
+        </is>
+      </c>
+      <c r="E7" s="2" t="inlineStr">
+        <is>
+          <t>Client required money to never be stuck; retry added complexity without guaranteeing fund safety</t>
+        </is>
+      </c>
+      <c r="F7" s="2" t="inlineStr">
+        <is>
+          <t>Retry feature fully removed; rollback/refund + 3-stage audit history (initiated/refunded/completed) added instead</t>
+        </is>
+      </c>
+      <c r="G7" s="2" t="inlineStr">
+        <is>
+          <t>Dhruv</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="2" t="inlineStr">
+        <is>
+          <t>DEC-07</t>
+        </is>
+      </c>
+      <c r="B8" s="2" t="inlineStr">
+        <is>
+          <t>Sprint 4</t>
+        </is>
+      </c>
+      <c r="C8" s="2" t="inlineStr">
+        <is>
+          <t>04-Aug-2026</t>
+        </is>
+      </c>
+      <c r="D8" s="2" t="inlineStr">
+        <is>
+          <t>Isolate password-change feature into its own branch/commit after a revert</t>
+        </is>
+      </c>
+      <c r="E8" s="2" t="inlineStr">
+        <is>
+          <t>First attempt was reverted due to it being bundled with unrelated changes; re-added cleanly on its own</t>
+        </is>
+      </c>
+      <c r="F8" s="2" t="inlineStr">
+        <is>
+          <t>Cleaner git history; AccountController/PasswordService added as a standalone, reviewable feature</t>
+        </is>
+      </c>
+      <c r="G8" s="2" t="inlineStr">
+        <is>
+          <t>Anusree</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="2" t="inlineStr">
+        <is>
+          <t>DEC-08</t>
+        </is>
+      </c>
+      <c r="B9" s="2" t="inlineStr">
+        <is>
+          <t>Sprint 5</t>
+        </is>
+      </c>
+      <c r="C9" s="2" t="inlineStr">
+        <is>
+          <t>05-Aug-2026</t>
+        </is>
+      </c>
+      <c r="D9" s="2" t="inlineStr">
+        <is>
+          <t>Use GitHub Actions (not Jenkins) for CI/CD</t>
+        </is>
+      </c>
+      <c r="E9" s="2" t="inlineStr">
+        <is>
+          <t>GitHub-native, zero infra to host/maintain, sufficient for build+test+docker-build at this project scale</t>
+        </is>
+      </c>
+      <c r="F9" s="2" t="inlineStr">
+        <is>
+          <t>ci.yml covers build-backend, build-frontend, and docker-build jobs; no self-hosted CI server needed</t>
+        </is>
+      </c>
+      <c r="G9" s="2" t="inlineStr">
+        <is>
+          <t>Dhruv</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:F4"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>